<commit_message>
Prompt 8: Colonnes EtatFi et Compta N/N-1 distinctes
mapping_parser.from_fm lit les colonnes K/L/M/N du FM (etatfi_n, etatfi_n1,
compta_n, compta_n1), cycle_mapper propage les 4 champs (aliases etatfi/compta
conservés ; comptes hors FM : N-1 vide, pas d'historique inventé),
fm_writer._ecrire_balance_tab écrit les 4 colonnes distinctes. GILAC : 22
comptes reclassés EtatFi, 23 Compta (413000, 421000, 425000...). Fixture
régénérée après vérification (diff limité aux colonnes L/N, 0 cellule
numérique). 2 assertions structurelles de test_cycle_mapper.py mises à jour
(ancienne structure 4 colonnes codée en dur). 213 tests verts (+13).

https://claude.ai/code/session_01Y7QNqKSGJocuCSBWFjyzu7
</commit_message>
<xml_diff>
--- a/tests/fixtures/FM_GILAC_2025_POST_FIX.xlsx
+++ b/tests/fixtures/FM_GILAC_2025_POST_FIX.xlsx
@@ -9689,11 +9689,7 @@
           <t>Passif</t>
         </is>
       </c>
-      <c r="N13" s="7" t="inlineStr">
-        <is>
-          <t>Passif</t>
-        </is>
-      </c>
+      <c r="N13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="7" t="inlineStr">
@@ -10873,11 +10869,7 @@
           <t>Actif</t>
         </is>
       </c>
-      <c r="N35" s="7" t="inlineStr">
-        <is>
-          <t>Actif</t>
-        </is>
-      </c>
+      <c r="N35" s="7" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="B36" s="7" t="inlineStr">
@@ -12543,11 +12535,7 @@
           <t>Passif</t>
         </is>
       </c>
-      <c r="N66" s="7" t="inlineStr">
-        <is>
-          <t>Passif</t>
-        </is>
-      </c>
+      <c r="N66" s="7" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="B67" s="7" t="inlineStr">
@@ -12591,11 +12579,7 @@
           <t>Passif</t>
         </is>
       </c>
-      <c r="N67" s="7" t="inlineStr">
-        <is>
-          <t>Passif</t>
-        </is>
-      </c>
+      <c r="N67" s="7" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="B68" s="7" t="inlineStr">
@@ -12693,11 +12677,7 @@
           <t>Actif</t>
         </is>
       </c>
-      <c r="N69" s="7" t="inlineStr">
-        <is>
-          <t>Actif</t>
-        </is>
-      </c>
+      <c r="N69" s="7" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="B70" s="7" t="inlineStr">
@@ -12795,11 +12775,7 @@
           <t>Actif</t>
         </is>
       </c>
-      <c r="N71" s="7" t="inlineStr">
-        <is>
-          <t>Actif</t>
-        </is>
-      </c>
+      <c r="N71" s="7" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="B72" s="7" t="inlineStr">
@@ -12843,11 +12819,7 @@
           <t>Actif</t>
         </is>
       </c>
-      <c r="N72" s="7" t="inlineStr">
-        <is>
-          <t>Actif</t>
-        </is>
-      </c>
+      <c r="N72" s="7" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="B73" s="7" t="inlineStr">
@@ -12889,7 +12861,7 @@
       </c>
       <c r="L73" s="7" t="inlineStr">
         <is>
-          <t>Clients et comptes rattachés</t>
+          <t>Clients créditeurs</t>
         </is>
       </c>
       <c r="M73" s="7" t="inlineStr">
@@ -12899,7 +12871,7 @@
       </c>
       <c r="N73" s="7" t="inlineStr">
         <is>
-          <t>Actif</t>
+          <t>Passif</t>
         </is>
       </c>
     </row>
@@ -13051,7 +13023,7 @@
       </c>
       <c r="L76" s="7" t="inlineStr">
         <is>
-          <t>Dettes sociales</t>
+          <t>Créances sociales</t>
         </is>
       </c>
       <c r="M76" s="7" t="inlineStr">
@@ -13061,7 +13033,7 @@
       </c>
       <c r="N76" s="7" t="inlineStr">
         <is>
-          <t>Passif</t>
+          <t>Actif</t>
         </is>
       </c>
     </row>
@@ -13105,7 +13077,7 @@
       </c>
       <c r="L77" s="7" t="inlineStr">
         <is>
-          <t>Dettes sociales</t>
+          <t>Créances sociales</t>
         </is>
       </c>
       <c r="M77" s="7" t="inlineStr">
@@ -13115,7 +13087,7 @@
       </c>
       <c r="N77" s="7" t="inlineStr">
         <is>
-          <t>Passif</t>
+          <t>Actif</t>
         </is>
       </c>
     </row>
@@ -13161,7 +13133,7 @@
       </c>
       <c r="L78" s="7" t="inlineStr">
         <is>
-          <t>Créances sociales</t>
+          <t>Dettes sociales</t>
         </is>
       </c>
       <c r="M78" s="7" t="inlineStr">
@@ -13171,7 +13143,7 @@
       </c>
       <c r="N78" s="7" t="inlineStr">
         <is>
-          <t>Actif</t>
+          <t>Passif</t>
         </is>
       </c>
     </row>
@@ -13269,7 +13241,7 @@
       </c>
       <c r="L80" s="7" t="inlineStr">
         <is>
-          <t>Dettes sociales</t>
+          <t>Créances sociales</t>
         </is>
       </c>
       <c r="M80" s="7" t="inlineStr">
@@ -13279,7 +13251,7 @@
       </c>
       <c r="N80" s="7" t="inlineStr">
         <is>
-          <t>Passif</t>
+          <t>Actif</t>
         </is>
       </c>
     </row>
@@ -13323,7 +13295,7 @@
       </c>
       <c r="L81" s="7" t="inlineStr">
         <is>
-          <t>Créances sociales</t>
+          <t>Dettes sociales</t>
         </is>
       </c>
       <c r="M81" s="7" t="inlineStr">
@@ -13333,7 +13305,7 @@
       </c>
       <c r="N81" s="7" t="inlineStr">
         <is>
-          <t>Actif</t>
+          <t>Passif</t>
         </is>
       </c>
     </row>
@@ -13701,7 +13673,7 @@
       </c>
       <c r="L88" s="7" t="inlineStr">
         <is>
-          <t>Dettes sociales</t>
+          <t>Créances sociales</t>
         </is>
       </c>
       <c r="M88" s="7" t="inlineStr">
@@ -13711,7 +13683,7 @@
       </c>
       <c r="N88" s="7" t="inlineStr">
         <is>
-          <t>Passif</t>
+          <t>Actif</t>
         </is>
       </c>
     </row>
@@ -13809,7 +13781,7 @@
       </c>
       <c r="L90" s="7" t="inlineStr">
         <is>
-          <t>Dettes sociales</t>
+          <t>Créances sociales</t>
         </is>
       </c>
       <c r="M90" s="7" t="inlineStr">
@@ -13819,7 +13791,7 @@
       </c>
       <c r="N90" s="7" t="inlineStr">
         <is>
-          <t>Passif</t>
+          <t>Actif</t>
         </is>
       </c>
     </row>
@@ -13971,7 +13943,7 @@
       </c>
       <c r="L93" s="7" t="inlineStr">
         <is>
-          <t>Créances fiscales</t>
+          <t>Dettes fiscales</t>
         </is>
       </c>
       <c r="M93" s="7" t="inlineStr">
@@ -13981,7 +13953,7 @@
       </c>
       <c r="N93" s="7" t="inlineStr">
         <is>
-          <t>Actif</t>
+          <t>Passif</t>
         </is>
       </c>
     </row>
@@ -14135,11 +14107,7 @@
           <t>Passif</t>
         </is>
       </c>
-      <c r="N96" s="7" t="inlineStr">
-        <is>
-          <t>Passif</t>
-        </is>
-      </c>
+      <c r="N96" s="7" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="B97" s="7" t="inlineStr">
@@ -14239,7 +14207,7 @@
       </c>
       <c r="L98" s="7" t="inlineStr">
         <is>
-          <t>Créances fiscales</t>
+          <t>Dettes fiscales</t>
         </is>
       </c>
       <c r="M98" s="7" t="inlineStr">
@@ -14249,7 +14217,7 @@
       </c>
       <c r="N98" s="7" t="inlineStr">
         <is>
-          <t>Actif</t>
+          <t>Passif</t>
         </is>
       </c>
     </row>
@@ -14571,7 +14539,7 @@
       </c>
       <c r="L104" s="7" t="inlineStr">
         <is>
-          <t>Créances fiscales</t>
+          <t>Dettes fiscales</t>
         </is>
       </c>
       <c r="M104" s="7" t="inlineStr">
@@ -14581,7 +14549,7 @@
       </c>
       <c r="N104" s="7" t="inlineStr">
         <is>
-          <t>Actif</t>
+          <t>Passif</t>
         </is>
       </c>
     </row>
@@ -14681,7 +14649,7 @@
       </c>
       <c r="L106" s="7" t="inlineStr">
         <is>
-          <t>Créances fiscales</t>
+          <t>Dettes fiscales</t>
         </is>
       </c>
       <c r="M106" s="7" t="inlineStr">
@@ -14691,7 +14659,7 @@
       </c>
       <c r="N106" s="7" t="inlineStr">
         <is>
-          <t>Actif</t>
+          <t>Passif</t>
         </is>
       </c>
     </row>
@@ -14735,7 +14703,7 @@
       </c>
       <c r="L107" s="7" t="inlineStr">
         <is>
-          <t>Emprunts et dettes financières</t>
+          <t>Comptes courants débiteurs</t>
         </is>
       </c>
       <c r="M107" s="7" t="inlineStr">
@@ -14745,7 +14713,7 @@
       </c>
       <c r="N107" s="7" t="inlineStr">
         <is>
-          <t>Passif</t>
+          <t>Actif</t>
         </is>
       </c>
     </row>
@@ -14789,7 +14757,7 @@
       </c>
       <c r="L108" s="7" t="inlineStr">
         <is>
-          <t>Emprunts et dettes financières</t>
+          <t>Comptes courants débiteurs</t>
         </is>
       </c>
       <c r="M108" s="7" t="inlineStr">
@@ -14799,7 +14767,7 @@
       </c>
       <c r="N108" s="7" t="inlineStr">
         <is>
-          <t>Passif</t>
+          <t>Actif</t>
         </is>
       </c>
     </row>
@@ -14843,7 +14811,7 @@
       </c>
       <c r="L109" s="7" t="inlineStr">
         <is>
-          <t>Emprunts et dettes financières</t>
+          <t>Comptes courants débiteurs</t>
         </is>
       </c>
       <c r="M109" s="7" t="inlineStr">
@@ -14853,7 +14821,7 @@
       </c>
       <c r="N109" s="7" t="inlineStr">
         <is>
-          <t>Passif</t>
+          <t>Actif</t>
         </is>
       </c>
     </row>
@@ -14951,7 +14919,7 @@
       </c>
       <c r="L111" s="7" t="inlineStr">
         <is>
-          <t>Emprunts et dettes financières</t>
+          <t>Comptes courants débiteurs</t>
         </is>
       </c>
       <c r="M111" s="7" t="inlineStr">
@@ -14961,7 +14929,7 @@
       </c>
       <c r="N111" s="7" t="inlineStr">
         <is>
-          <t>Passif</t>
+          <t>Actif</t>
         </is>
       </c>
     </row>
@@ -15059,7 +15027,7 @@
       </c>
       <c r="L113" s="7" t="inlineStr">
         <is>
-          <t>Emprunts et dettes financières</t>
+          <t>Comptes courants débiteurs</t>
         </is>
       </c>
       <c r="M113" s="7" t="inlineStr">
@@ -15069,7 +15037,7 @@
       </c>
       <c r="N113" s="7" t="inlineStr">
         <is>
-          <t>Passif</t>
+          <t>Actif</t>
         </is>
       </c>
     </row>
@@ -15115,11 +15083,7 @@
           <t>Passif</t>
         </is>
       </c>
-      <c r="N114" s="7" t="inlineStr">
-        <is>
-          <t>Passif</t>
-        </is>
-      </c>
+      <c r="N114" s="7" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="B115" s="7" t="inlineStr">
@@ -15161,7 +15125,7 @@
       </c>
       <c r="L115" s="7" t="inlineStr">
         <is>
-          <t>Emprunts et dettes financières</t>
+          <t>Comptes courants débiteurs</t>
         </is>
       </c>
       <c r="M115" s="7" t="inlineStr">
@@ -15171,7 +15135,7 @@
       </c>
       <c r="N115" s="7" t="inlineStr">
         <is>
-          <t>Passif</t>
+          <t>Actif</t>
         </is>
       </c>
     </row>
@@ -15323,7 +15287,7 @@
       </c>
       <c r="L118" s="7" t="inlineStr">
         <is>
-          <t>Créances diverses</t>
+          <t>Dettes diverses</t>
         </is>
       </c>
       <c r="M118" s="7" t="inlineStr">
@@ -15333,7 +15297,7 @@
       </c>
       <c r="N118" s="7" t="inlineStr">
         <is>
-          <t>Actif</t>
+          <t>Passif</t>
         </is>
       </c>
     </row>
@@ -15433,11 +15397,7 @@
           <t>Actif</t>
         </is>
       </c>
-      <c r="N120" s="7" t="inlineStr">
-        <is>
-          <t>Actif</t>
-        </is>
-      </c>
+      <c r="N120" s="7" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="B121" s="7" t="inlineStr">
@@ -15589,7 +15549,7 @@
       </c>
       <c r="L123" s="7" t="inlineStr">
         <is>
-          <t>Emprunts et dettes auprès d'établissements de crédit</t>
+          <t>Disponibilités</t>
         </is>
       </c>
       <c r="M123" s="7" t="inlineStr">
@@ -15599,7 +15559,7 @@
       </c>
       <c r="N123" s="7" t="inlineStr">
         <is>
-          <t>Passif</t>
+          <t>Actif</t>
         </is>
       </c>
     </row>
@@ -15753,11 +15713,7 @@
           <t>Actif</t>
         </is>
       </c>
-      <c r="N126" s="7" t="inlineStr">
-        <is>
-          <t>Actif</t>
-        </is>
-      </c>
+      <c r="N126" s="7" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="B127" s="7" t="inlineStr">
@@ -16071,11 +16027,7 @@
           <t>Actif</t>
         </is>
       </c>
-      <c r="N132" s="7" t="inlineStr">
-        <is>
-          <t>Actif</t>
-        </is>
-      </c>
+      <c r="N132" s="7" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="B133" s="7" t="inlineStr">
@@ -16119,11 +16071,7 @@
           <t>Actif</t>
         </is>
       </c>
-      <c r="N133" s="7" t="inlineStr">
-        <is>
-          <t>Actif</t>
-        </is>
-      </c>
+      <c r="N133" s="7" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="B134" s="7" t="inlineStr">
@@ -16817,11 +16765,7 @@
           <t>Charges</t>
         </is>
       </c>
-      <c r="N146" s="7" t="inlineStr">
-        <is>
-          <t>Charges</t>
-        </is>
-      </c>
+      <c r="N146" s="7" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="B147" s="7" t="inlineStr">
@@ -17351,11 +17295,7 @@
           <t>Charges</t>
         </is>
       </c>
-      <c r="N156" s="7" t="inlineStr">
-        <is>
-          <t>Charges</t>
-        </is>
-      </c>
+      <c r="N156" s="7" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="B157" s="7" t="inlineStr">
@@ -17877,11 +17817,7 @@
           <t>Charges</t>
         </is>
       </c>
-      <c r="N166" s="7" t="inlineStr">
-        <is>
-          <t>Charges</t>
-        </is>
-      </c>
+      <c r="N166" s="7" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="B167" s="7" t="inlineStr">
@@ -18897,11 +18833,7 @@
           <t>Charges</t>
         </is>
       </c>
-      <c r="N185" s="7" t="inlineStr">
-        <is>
-          <t>Charges</t>
-        </is>
-      </c>
+      <c r="N185" s="7" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="B186" s="7" t="inlineStr">
@@ -19161,11 +19093,7 @@
           <t>Charges</t>
         </is>
       </c>
-      <c r="N190" s="7" t="inlineStr">
-        <is>
-          <t>Charges</t>
-        </is>
-      </c>
+      <c r="N190" s="7" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="B191" s="7" t="inlineStr">
@@ -19425,11 +19353,7 @@
           <t>Charges</t>
         </is>
       </c>
-      <c r="N195" s="7" t="inlineStr">
-        <is>
-          <t>Charges</t>
-        </is>
-      </c>
+      <c r="N195" s="7" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="B196" s="7" t="inlineStr">
@@ -19689,11 +19613,7 @@
           <t>Charges</t>
         </is>
       </c>
-      <c r="N200" s="7" t="inlineStr">
-        <is>
-          <t>Charges</t>
-        </is>
-      </c>
+      <c r="N200" s="7" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="B201" s="7" t="inlineStr">
@@ -19737,11 +19657,7 @@
           <t>Charges</t>
         </is>
       </c>
-      <c r="N201" s="7" t="inlineStr">
-        <is>
-          <t>Charges</t>
-        </is>
-      </c>
+      <c r="N201" s="7" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="B202" s="7" t="inlineStr">
@@ -20973,11 +20889,7 @@
           <t>Charges</t>
         </is>
       </c>
-      <c r="N224" s="7" t="inlineStr">
-        <is>
-          <t>Charges</t>
-        </is>
-      </c>
+      <c r="N224" s="7" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="B225" s="7" t="inlineStr">
@@ -21237,11 +21149,7 @@
           <t>Charges</t>
         </is>
       </c>
-      <c r="N229" s="7" t="inlineStr">
-        <is>
-          <t>Charges</t>
-        </is>
-      </c>
+      <c r="N229" s="7" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="B230" s="7" t="inlineStr">
@@ -21991,11 +21899,7 @@
           <t>Charges</t>
         </is>
       </c>
-      <c r="N243" s="7" t="inlineStr">
-        <is>
-          <t>Charges</t>
-        </is>
-      </c>
+      <c r="N243" s="7" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="B244" s="7" t="inlineStr">
@@ -22257,11 +22161,7 @@
           <t>Charges</t>
         </is>
       </c>
-      <c r="N248" s="7" t="inlineStr">
-        <is>
-          <t>Charges</t>
-        </is>
-      </c>
+      <c r="N248" s="7" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="B249" s="7" t="inlineStr">
@@ -23655,11 +23555,7 @@
           <t>Produits</t>
         </is>
       </c>
-      <c r="N274" s="7" t="inlineStr">
-        <is>
-          <t>Produits</t>
-        </is>
-      </c>
+      <c r="N274" s="7" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="B275" s="7" t="inlineStr">
@@ -23703,11 +23599,7 @@
           <t>Produits</t>
         </is>
       </c>
-      <c r="N275" s="7" t="inlineStr">
-        <is>
-          <t>Produits</t>
-        </is>
-      </c>
+      <c r="N275" s="7" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="B276" s="7" t="inlineStr">
@@ -23805,11 +23697,7 @@
           <t>Produits</t>
         </is>
       </c>
-      <c r="N277" s="7" t="inlineStr">
-        <is>
-          <t>Produits</t>
-        </is>
-      </c>
+      <c r="N277" s="7" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="B278" s="7" t="inlineStr">
@@ -23853,11 +23741,7 @@
           <t>Produits</t>
         </is>
       </c>
-      <c r="N278" s="7" t="inlineStr">
-        <is>
-          <t>Produits</t>
-        </is>
-      </c>
+      <c r="N278" s="7" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="B279" s="7" t="inlineStr">

</xml_diff>